<commit_message>
feat: traducción completa del Disco 1 (299 escenas)
</commit_message>
<xml_diff>
--- a/translation/review/000scriptAKYO_0000A.xlsx
+++ b/translation/review/000scriptAKYO_0000A.xlsx
@@ -22,25 +22,25 @@
     <t>My little sister's name is Kousaka Kirino, and she attends the nearby middle school.</t>
   </si>
   <si>
-    <t>El nombre de mi hermanita es Kousaka Kirino, y va a la secundaria de aquí al lado.</t>
+    <t>El nombre de mi hermanita es Kousaka Kirino, y＿va a la secundaria de aquí al lado.</t>
   </si>
   <si>
     <t>With auburn dyed hair, both ears pierced, and her long manicured nails...</t>
   </si>
   <si>
-    <t>Con el pelo teñido de castaño, ambas orejas perforadas y sus uñas largas y cuidadas...</t>
+    <t>Con el pelo teñido de castaño, ambas orejas＿perforadas y sus uñas largas y cuidadas...</t>
   </si>
   <si>
     <t>Her pretty face draws enough attention even without makeup; but with it, she's absolutely stunning!</t>
   </si>
   <si>
-    <t>Su bonita cara llama la atención incluso sin maquillaje; ¡pero con él, está absolutamente impresionante!</t>
+    <t>Su bonita cara llama la atención incluso sin＿maquillaje; ¡pero con él, está absolutamente＿impresionante!</t>
   </si>
   <si>
     <t>She has a rare mature look for a middle schooler; although her face is slightly roundish.</t>
   </si>
   <si>
-    <t>Tiene una madurez poco común para una chica de secundaria; aunque su rostro es un poco redondeado.</t>
+    <t>Tiene una madurez poco común para una chica de＿secundaria; aunque su rostro es un poco＿redondeado.</t>
   </si>
   <si>
     <t>Anyway, my little sister is an outstanding girl.</t>
@@ -52,13 +52,13 @@
     <t>Furthermore, she's a model for a teen magazine, the ace of the track and field club, and ranked fifth in academic tests...</t>
   </si>
   <si>
-    <t>Además, es modelo de una revista juvenil, la estrella del club de atletismo y ocupa el quinto lugar en los exámenes...</t>
+    <t>Además, es modelo de una revista juvenil, la＿estrella del club de atletismo y ocupa el quinto＿lugar en los exámenes...</t>
   </si>
   <si>
     <t>In school, there's always that group of glamorous students with whom it's hard to start a conversation with, right?</t>
   </si>
   <si>
-    <t>En la escuela siempre existe ese grupo de estudiantes glamorosos con los que es difícil entablar una conversación, ¿verdad?</t>
+    <t>En la escuela siempre existe ese grupo de＿estudiantes glamorosos con los que es difícil＿entablar una conversación, ¿verdad?</t>
   </si>
   <si>
     <t>Well, the core of that group is Kirino.</t>
@@ -76,19 +76,19 @@
     <t>...How was it? Now do you understand my embarrassment slightly better?</t>
   </si>
   <si>
-    <t>...¿Y qué? ¿Ahora entiendes un poco mejor mi vergüenza?</t>
+    <t>...¿Y qué? ¿Ahora entiendes un poco mejor mi＿vergüenza?</t>
   </si>
   <si>
     <t>With that, my name is Kousaka Kyousuke. I am eighteen years old, attending the nearby high school.</t>
   </si>
   <si>
-    <t>Dicho esto, mi nombre es Kousaka Kyousuke. Tengo dieciocho años y asisto a la preparatoria de aquí al lado.</t>
+    <t>Dicho esto, mi nombre es Kousaka Kyousuke.＿Tengo dieciocho años y asisto a la preparatoria＿de aquí al lado.</t>
   </si>
   <si>
     <t>Although it's a little embarrassing, I'm a very ordinary high school student...</t>
   </si>
   <si>
-    <t>Aunque sea un poco vergonzoso, soy un estudiante de preparatoria muy común...</t>
+    <t>Aunque sea un poco vergonzoso, soy un＿estudiante de preparatoria muy común...</t>
   </si>
   <si>
     <t>Only wishing to live a normal life.</t>
@@ -100,31 +100,31 @@
     <t>Neither being involved in daily situations that are far out of the ordinary, nor meeting unique people is needed in my life.</t>
   </si>
   <si>
-    <t>No necesito en mi vida situaciones cotidianas fuera de lo común ni conocer gente peculiar.</t>
+    <t>No necesito en mi vida situaciones cotidianas＿fuera de lo común ni conocer gente peculiar.</t>
   </si>
   <si>
     <t>You might say that I'm a slacker, but mediocrity is my motto.</t>
   </si>
   <si>
-    <t>Podrías decir que soy un holgazán, pero la mediocridad es mi lema.</t>
+    <t>Podrías decir que soy un holgazán, pero la＿mediocridad es mi lema.</t>
   </si>
   <si>
     <t>My goal is to watch the never-changing, stagnating scenery.</t>
   </si>
   <si>
-    <t>Mi meta es contemplar el paisaje inmutable y estancado.</t>
+    <t>Mi meta es contemplar el paisaje inmutable y＿estancado.</t>
   </si>
   <si>
     <t>Mediocrity banzai! Viva my ordinary life... Or so it should be...</t>
   </si>
   <si>
-    <t>¡Banzai a la mediocridad! ¡Viva mi vida ordinaria...! O eso debería ser...</t>
+    <t>¡Banzai a la mediocridad! ¡Viva mi vida ordinaria...!＿O eso debería ser...</t>
   </si>
   <si>
     <t>If only I didn't get involved with my sister and the "pleasant comrades" surrounding her...</t>
   </si>
   <si>
-    <t>Si tan solo no me hubiera involucrado con mi hermana y los «agradables camaradas» que la rodean...</t>
+    <t>Si tan solo no me hubiera involucrado con mi＿hermana y los «agradables camaradas» que la＿rodean...</t>
   </si>
   <si>
     <t>Kirino</t>
@@ -145,7 +145,7 @@
     <t>The perfect beautiful middle schooler in my eyes is actually...</t>
   </si>
   <si>
-    <t>La chica de secundaria perfecta y hermosa ante mis ojos es en realidad...</t>
+    <t>La chica de secundaria perfecta y hermosa ante＿mis ojos es en realidad...</t>
   </si>
   <si>
     <t>Kyousuke</t>
@@ -154,7 +154,7 @@
     <t>...So you mean, you, erm... Though it's hard to believe...</t>
   </si>
   <si>
-    <t>...Entonces quieres decir que tú, eh... Aunque sea difícil de creer...</t>
+    <t>...Entonces quieres decir que tú, eh... Aunque＿sea difícil de creer...</t>
   </si>
   <si>
     <t>You like "little sisters"?</t>
@@ -178,7 +178,7 @@
     <t>Having a large quantity of little sister related games... an otaku.</t>
   </si>
   <si>
-    <t>Tener una gran cantidad de juegos relacionados con hermanitas... una otaku.</t>
+    <t>Tener una gran cantidad de juegos relacionados＿con hermanitas... una otaku.</t>
   </si>
   <si>
     <t>For future reference, I must say this...</t>
@@ -190,7 +190,7 @@
     <t>If anyone were to ask you for a "life counseling session", it would be better to reject it.</t>
   </si>
   <si>
-    <t>Si alguien te pidiera una «sesión de orientación en la vida», sería mejor que la rechazaras.</t>
+    <t>Si alguien te pidiera una «sesión de orientación en＿la vida», sería mejor que la rechazaras.</t>
   </si>
   <si>
     <t>Especially if that person is your "little sister".</t>
@@ -202,7 +202,7 @@
     <t>If that little sister holds anime DVDs and games unfit for children in her hands, it's best to hit the road at once.</t>
   </si>
   <si>
-    <t>Si esa hermanita tiene entre manos DVDs de anime y juegos no aptos para niños, lo mejor es salir corriendo de inmediato.</t>
+    <t>Si esa hermanita tiene entre manos DVDs de＿anime y juegos no aptos para niños, lo mejor es＿salir corriendo de inmediato.</t>
   </si>
   <si>
     <t>If not...</t>
@@ -223,7 +223,7 @@
     <t>Welcome home, Onii-chan! Let's make love... together with your little sister～</t>
   </si>
   <si>
-    <t>¡Bienvenido a casa, Onii-chan! Hagamos el amor... junto con tu hermanita～</t>
+    <t>¡Bienvenido a casa, Onii-chan! Hagamos el＿amor... junto con tu hermanita～</t>
   </si>
   <si>
     <t>The heck are you trying to make me play!?!</t>
@@ -235,7 +235,7 @@
     <t>Being forced to play games I don't want to, night after night...</t>
   </si>
   <si>
-    <t>Obligado a jugar juegos que no quiero, noche tras noche...</t>
+    <t>Obligado a jugar juegos que no quiero, noche tras＿noche...</t>
   </si>
   <si>
     <t>...Hey, what do you think I should do?</t>
@@ -247,13 +247,13 @@
     <t>Make some friends, people with the same hobbies as you should do.</t>
   </si>
   <si>
-    <t>Hazte amigos, gente con los mismos gustos que tú, como deberías hacer.</t>
+    <t>Hazte amigos, gente con los mismos gustos＿que tú, como deberías hacer.</t>
   </si>
   <si>
     <t>Working herself up over her ability to make like-minded friends...</t>
   </si>
   <si>
-    <t>Enfadándose por su capacidad para hacer amigos afines...</t>
+    <t>Enfadándose por su capacidad para hacer amigos＿afines...</t>
   </si>
   <si>
     <t>Saori</t>
@@ -286,7 +286,7 @@
     <t>...Oh, in other words - you were in your sister's room, using your sister's computer, and playing some game that does indecent things to sisters?</t>
   </si>
   <si>
-    <t>...Ah, o sea: estabas en el cuarto de tu hermana, usando su computadora y jugando un juego que hace cosas indecentes con las hermanitas?</t>
+    <t>...Ah, o sea: estabas en el cuarto de tu hermana,＿usando su computadora y jugando un juego＿que hace cosas indecentes con las hermanitas?</t>
   </si>
   <si>
     <t>They're super interesting! Any problem with that?!</t>
@@ -343,7 +343,7 @@
     <t>Radio Kaikan! AniMate! Huhu... So this is Akihabara!!</t>
   </si>
   <si>
-    <t>¡Radio Kaikan! ¡AniMate! Juju... ¡Así que esto es Akihabara!!</t>
+    <t>¡Radio Kaikan! ¡AniMate! Juju... ¡Así que esto es＿Akihabara!!</t>
   </si>
   <si>
     <t>It's really cute, isn't it? Erm, for example...</t>
@@ -355,37 +355,37 @@
     <t>Since a lot of galges are directed towards male players, there are salutations like 'Onii-chan', 'Onii', 'Aniki', 'Nii-kun'...</t>
   </si>
   <si>
-    <t>Como muchos galges están dirigidos a jugadores hombres, hay saludos como «Onii-chan», «Onii», «Aniki», «Nii-kun»...</t>
+    <t>Como muchos galges están dirigidos a＿jugadores hombres, hay saludos como＿«Onii-chan», «Onii», «Aniki», «Nii-kun»...</t>
   </si>
   <si>
     <t>The girls call me with whatever "special salutation" that fits their character, which shows their affection for me. It's simply... too CUTE!</t>
   </si>
   <si>
-    <t>Las chicas me llaman con el «saludo especial» que encaja con su personaje, lo que muestra su afecto hacia mí. ¡Es simplemente... demasiado LINDO!</t>
+    <t>Las chicas me llaman con el «saludo especial»＿que encaja con su personaje, lo que muestra[su afecto hacia mí. ¡Es simplemente...＿demasiado LINDO!]</t>
   </si>
   <si>
     <t>It's the Summer Comiket limited edition "Stardust ☆ Witch Meruru" dakimakura set! Isn't it awesome?</t>
   </si>
   <si>
-    <t>¡Es el set de dakimakura de edición limitada del Comiket de verano de «Stardust ☆ Witch Meruru»! ¿No es increíble?</t>
+    <t>¡Es el set de dakimakura de edición limitada del＿Comiket de verano de «Stardust ☆ Witch＿Meruru»! ¿No es increíble?</t>
   </si>
   <si>
     <t>Eh? It's a dakimakura, so of course you're supposed to hug it to sleep.</t>
   </si>
   <si>
-    <t>¿Eh? Es una dakimakura, así que por supuesto se supone que la abrazas para dormir.</t>
+    <t>¿Eh? Es una dakimakura, así que por supuesto＿se supone que la abrazas para dormir.</t>
   </si>
   <si>
     <t>Well, sometimes you rub your face against it, and maybe smell it...</t>
   </si>
   <si>
-    <t>Bueno, a veces restriegas la cara contra ella, y tal vez la hueles...</t>
+    <t>Bueno, a veces restriegas la cara contra ella, y＿tal vez la hueles...</t>
   </si>
   <si>
     <t>Looking at my sister happily fooling around with her hobby, I feel that it isn't all too bad.</t>
   </si>
   <si>
-    <t>Al ver a mi hermana disfrutando feliz de su pasatiempo, siento que no está tan mal.</t>
+    <t>Al ver a mi hermana disfrutando feliz de su＿pasatiempo, siento que no está tan mal.</t>
   </si>
   <si>
     <t>It must be because I'm her elder brother.</t>

</xml_diff>